<commit_message>
Independent check: 2 classmates agree on 10 of 10
</commit_message>
<xml_diff>
--- a/docs/evidence/myTutor_evidence_workbook.xlsx
+++ b/docs/evidence/myTutor_evidence_workbook.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="198">
   <si>
     <t xml:space="preserve">myTutor stretch evidence workbook</t>
   </si>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Second reviewer (optional, a subset)</t>
   </si>
   <si>
-    <t xml:space="preserve">None</t>
+    <t xml:space="preserve">Shawn (5 claims) and Faiiz (5 claims): classmates, blind, random draw of 10 of the 30 claims; all rated Supported</t>
   </si>
   <si>
     <t xml:space="preserve">Notes in sample</t>
@@ -190,7 +190,7 @@
     <t xml:space="preserve">Fix / prompt change</t>
   </si>
   <si>
-    <t xml:space="preserve">2nd reviewer agrees? (Y/N)</t>
+    <t xml:space="preserve">2nd reviewer agrees? (blind check)</t>
   </si>
   <si>
     <t xml:space="preserve">Case - Hewlett-Packard</t>
@@ -214,6 +214,9 @@
     <t xml:space="preserve">A small team several layers down built a handheld scanner prototype; flatbed-focused managers gave it no attention</t>
   </si>
   <si>
+    <t xml:space="preserve">Y (Shawn)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Antonio Perez intervened with $10 million to validate the portables business</t>
   </si>
   <si>
@@ -242,6 +245,9 @@
   </si>
   <si>
     <t xml:space="preserve">Note omits 2019 / Kevin Johnson; omission, not error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y (Faiiz)</t>
   </si>
   <si>
     <t xml:space="preserve">Case - USA Today</t>
@@ -790,7 +796,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -864,10 +870,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1418,8 +1420,8 @@
         <v>46</v>
       </c>
       <c r="H13" s="1" t="str">
-        <f aca="false">IF(H5=0,"","Manual self-audit (Day 10, by Naw Aung): "&amp;H6&amp;" of "&amp;H5&amp;" claims supported ("&amp;TEXT(H10,"0%")&amp;") across "&amp;H11&amp;" notes (3 case, 5 core) drawn at random by n8n, "&amp;H12&amp;" substantive errors; each checked against the source page. 2 quiz notes in the sample were excluded.")</f>
-        <v>Manual self-audit (Day 10, by Naw Aung): 30 of 30 claims supported (100%) across 8 notes (3 case, 5 core) drawn at random by n8n, 0 substantive errors; each checked against the source page. 2 quiz notes in the sample were excluded.</v>
+        <f aca="false">IF(H5=0,"","Manual self-audit (Day 10, by Naw Aung): "&amp;H6&amp;" of "&amp;H5&amp;" claims supported ("&amp;TEXT(H10,"0%")&amp;") across "&amp;H11&amp;" notes (3 case, 5 core) drawn at random by n8n, "&amp;H12&amp;" substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: "&amp;COUNTIF(J15:J44,"Y*")&amp;" of 10 agree. 2 quiz notes in the sample were excluded.")</f>
+        <v>Manual self-audit (Day 10, by Naw Aung): 30 of 30 claims supported (100%) across 8 notes (3 case, 5 core) drawn at random by n8n, 0 substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: 10 of 10 agree. 2 quiz notes in the sample were excluded.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1504,7 +1506,9 @@
       <c r="I16" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J16" s="7"/>
+      <c r="J16" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
@@ -1517,7 +1521,7 @@
         <v>58</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E17" s="7" t="s">
         <v>60</v>
@@ -1530,7 +1534,9 @@
       <c r="I17" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J17" s="7"/>
+      <c r="J17" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
@@ -1543,7 +1549,7 @@
         <v>58</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E18" s="7" t="s">
         <v>60</v>
@@ -1556,23 +1562,25 @@
       <c r="I18" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J18" s="7"/>
+      <c r="J18" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>28</v>
@@ -1586,19 +1594,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B20" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D20" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" s="7" t="s">
         <v>69</v>
-      </c>
-      <c r="E20" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>28</v>
@@ -1612,19 +1620,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B21" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E21" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>28</v>
@@ -1638,35 +1646,37 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B22" s="7" t="s">
         <v>57</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>28</v>
       </c>
       <c r="G22" s="7"/>
       <c r="H22" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J22" s="7"/>
+      <c r="J22" s="7" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>57</v>
@@ -1675,10 +1685,10 @@
         <v>58</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E23" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>28</v>
@@ -1692,7 +1702,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>57</v>
@@ -1701,10 +1711,10 @@
         <v>58</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E24" s="7" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>28</v>
@@ -1718,7 +1728,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>57</v>
@@ -1727,10 +1737,10 @@
         <v>58</v>
       </c>
       <c r="D25" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E25" s="7" t="s">
         <v>77</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>28</v>
@@ -1744,19 +1754,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C26" s="7" t="s">
         <v>58</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>28</v>
@@ -1770,47 +1780,49 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B27" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C27" s="7" t="s">
         <v>58</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="E27" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>28</v>
       </c>
       <c r="G27" s="7"/>
       <c r="H27" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J27" s="7"/>
+      <c r="J27" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>28</v>
@@ -1824,19 +1836,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B29" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E29" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>28</v>
@@ -1850,19 +1862,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D30" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E30" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="E30" s="7" t="s">
-        <v>88</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>28</v>
@@ -1876,19 +1888,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B31" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D31" s="7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E31" s="7" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>28</v>
@@ -1902,19 +1914,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B32" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>28</v>
@@ -1928,16 +1940,16 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B33" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E33" s="7" t="s">
         <v>60</v>
@@ -1954,16 +1966,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B34" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>60</v>
@@ -1980,16 +1992,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>60</v>
@@ -2002,20 +2014,22 @@
       <c r="I35" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J35" s="7"/>
+      <c r="J35" s="7" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>60</v>
@@ -2025,7 +2039,7 @@
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="7" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I36" s="7" t="s">
         <v>61</v>
@@ -2034,19 +2048,19 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>28</v>
@@ -2056,23 +2070,25 @@
       <c r="I37" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J37" s="7"/>
+      <c r="J37" s="7" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>28</v>
@@ -2082,30 +2098,32 @@
       <c r="I38" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J38" s="7"/>
+      <c r="J38" s="7" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>28</v>
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="I39" s="7" t="s">
         <v>61</v>
@@ -2114,19 +2132,19 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>28</v>
@@ -2136,23 +2154,25 @@
       <c r="I40" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J40" s="7"/>
+      <c r="J40" s="7" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>28</v>
@@ -2166,19 +2186,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>28</v>
@@ -2192,19 +2212,19 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D43" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E43" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="E43" s="7" t="s">
-        <v>111</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>28</v>
@@ -2218,19 +2238,19 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>28</v>
@@ -2240,7 +2260,9 @@
       <c r="I44" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="J44" s="7"/>
+      <c r="J44" s="7" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7"/>
@@ -4343,20 +4365,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
@@ -4368,10 +4390,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
@@ -4383,10 +4405,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
@@ -4398,10 +4420,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
@@ -4413,10 +4435,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
@@ -4428,57 +4450,57 @@
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>2061</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>0</v>
@@ -4498,27 +4520,27 @@
         <v>4.20669577874818</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>2360</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>1.02</v>
@@ -4538,27 +4560,27 @@
         <v>0.930084745762712</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>2077</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>0</v>
@@ -4578,27 +4600,27 @@
         <v>3.15358690418873</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>1578</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>1.02</v>
@@ -4618,10 +4640,10 @@
         <v>1.39100126742712</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4631,7 +4653,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">IFERROR((H11+H13)/(D11+D13)*1000,"")</f>
@@ -4640,7 +4662,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">IFERROR((H12+H14)/(D12+D14)*1000,"")</f>
@@ -4649,7 +4671,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B19" s="16" t="n">
         <f aca="false">IFERROR(1-B18/B17,"")</f>
@@ -4658,18 +4680,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>2.92</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>0.81</v>
@@ -4677,7 +4699,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B22" s="16" t="n">
         <f aca="false">1-B21/B20</f>
@@ -4732,105 +4754,105 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>175</v>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="L11" s="20" t="s">
-        <v>186</v>
-      </c>
-      <c r="M11" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="N11" s="20" t="s">
+      <c r="L11" s="19" t="s">
         <v>188</v>
+      </c>
+      <c r="M11" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="N11" s="19" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B12" s="6" t="n">
         <v>1</v>
@@ -4847,7 +4869,7 @@
       </c>
       <c r="J12" s="7"/>
       <c r="L12" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M12" s="8" t="n">
         <f aca="false">SUM(I12:I31)</f>
@@ -4860,7 +4882,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B13" s="6" t="n">
         <v>2</v>
@@ -4877,7 +4899,7 @@
       </c>
       <c r="J13" s="7"/>
       <c r="L13" s="6" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="M13" s="8" t="n">
         <f aca="false">SUM(G12:G31)</f>
@@ -4890,7 +4912,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>3</v>
@@ -4907,7 +4929,7 @@
       </c>
       <c r="J14" s="7"/>
       <c r="L14" s="6" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="M14" s="8" t="n">
         <f aca="false">SUM(H12:H31)</f>
@@ -4920,7 +4942,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B15" s="6" t="n">
         <v>4</v>
@@ -4937,7 +4959,7 @@
       </c>
       <c r="J15" s="7"/>
       <c r="L15" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="M15" s="8" t="n">
         <f aca="false">SUM(E12:E31)</f>
@@ -4950,7 +4972,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B16" s="6" t="n">
         <v>5</v>
@@ -4967,20 +4989,20 @@
       </c>
       <c r="J16" s="7"/>
       <c r="L16" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="M16" s="21" t="str">
+        <v>195</v>
+      </c>
+      <c r="M16" s="20" t="str">
         <f aca="false">IFERROR(COUNTIF(D12:D31,"B")/COUNTA(D12:D31),"")</f>
         <v/>
       </c>
-      <c r="N16" s="21" t="str">
+      <c r="N16" s="20" t="str">
         <f aca="false">IFERROR(COUNTIF(D32:D51,"B")/COUNTA(D32:D51),"")</f>
         <v/>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B17" s="6" t="n">
         <v>6</v>
@@ -4997,7 +5019,7 @@
       </c>
       <c r="J17" s="7"/>
       <c r="L17" s="6" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="M17" s="8" t="n">
         <f aca="false">COUNT(I12:I31)</f>
@@ -5010,7 +5032,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>7</v>
@@ -5027,20 +5049,20 @@
       </c>
       <c r="J18" s="7"/>
       <c r="L18" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="M18" s="21" t="str">
+        <v>197</v>
+      </c>
+      <c r="M18" s="20" t="str">
         <f aca="false">IFERROR(M12/(M17*5),"")</f>
         <v/>
       </c>
-      <c r="N18" s="21" t="str">
+      <c r="N18" s="20" t="str">
         <f aca="false">IFERROR(N12/(N17*5),"")</f>
         <v/>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>8</v>
@@ -5059,7 +5081,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>9</v>
@@ -5081,7 +5103,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>10</v>
@@ -5104,7 +5126,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B22" s="6" t="n">
         <v>11</v>
@@ -5123,7 +5145,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B23" s="6" t="n">
         <v>12</v>
@@ -5142,7 +5164,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B24" s="6" t="n">
         <v>13</v>
@@ -5161,7 +5183,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B25" s="6" t="n">
         <v>14</v>
@@ -5180,7 +5202,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B26" s="6" t="n">
         <v>15</v>
@@ -5199,7 +5221,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B27" s="6" t="n">
         <v>16</v>
@@ -5218,7 +5240,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B28" s="6" t="n">
         <v>17</v>
@@ -5237,7 +5259,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B29" s="6" t="n">
         <v>18</v>
@@ -5256,7 +5278,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B30" s="6" t="n">
         <v>19</v>
@@ -5275,7 +5297,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B31" s="6" t="n">
         <v>20</v>
@@ -5294,7 +5316,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B32" s="6" t="n">
         <v>1</v>
@@ -5313,7 +5335,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B33" s="6" t="n">
         <v>2</v>
@@ -5332,7 +5354,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B34" s="6" t="n">
         <v>3</v>
@@ -5351,7 +5373,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B35" s="6" t="n">
         <v>4</v>
@@ -5370,7 +5392,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B36" s="6" t="n">
         <v>5</v>
@@ -5389,7 +5411,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B37" s="6" t="n">
         <v>6</v>
@@ -5408,7 +5430,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B38" s="6" t="n">
         <v>7</v>
@@ -5427,7 +5449,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B39" s="6" t="n">
         <v>8</v>
@@ -5446,7 +5468,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B40" s="6" t="n">
         <v>9</v>
@@ -5465,7 +5487,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B41" s="6" t="n">
         <v>10</v>
@@ -5484,7 +5506,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B42" s="6" t="n">
         <v>11</v>
@@ -5503,7 +5525,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B43" s="6" t="n">
         <v>12</v>
@@ -5522,7 +5544,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B44" s="6" t="n">
         <v>13</v>
@@ -5541,7 +5563,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B45" s="6" t="n">
         <v>14</v>
@@ -5560,7 +5582,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B46" s="6" t="n">
         <v>15</v>
@@ -5579,7 +5601,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B47" s="6" t="n">
         <v>16</v>
@@ -5598,7 +5620,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B48" s="6" t="n">
         <v>17</v>
@@ -5617,7 +5639,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B49" s="6" t="n">
         <v>18</v>
@@ -5636,7 +5658,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B50" s="6" t="n">
         <v>19</v>
@@ -5655,7 +5677,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B51" s="6" t="n">
         <v>20</v>

</xml_diff>

<commit_message>
Version 4.1: final deck
</commit_message>
<xml_diff>
--- a/docs/evidence/myTutor_evidence_workbook.xlsx
+++ b/docs/evidence/myTutor_evidence_workbook.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="199">
   <si>
     <t xml:space="preserve">myTutor stretch evidence workbook</t>
   </si>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">Second reviewer (optional, a subset)</t>
   </si>
   <si>
-    <t xml:space="preserve">Shawn (5 claims) and Faiiz (5 claims): classmates, blind, random draw of 10 of the 30 claims; all rated Supported</t>
+    <t xml:space="preserve">Shawn and Faiiz (classmates) each independently checked 5 different claims (random draw of 10 of 30) against the original sources, without seeing my ratings. Shawn 5/5 Supported; Faiiz 4/5 Supported, 1 Interpretation (teleology definition). Agreement 9/10. Confirmations retained by email.</t>
   </si>
   <si>
     <t xml:space="preserve">Notes in sample</t>
@@ -337,6 +337,9 @@
     <t xml:space="preserve">PDF p. 2, col. 2</t>
   </si>
   <si>
+    <t xml:space="preserve">N (Faiiz: Interpretation; "purpose" is the note's gloss)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Epistemology asks what counts as knowledge</t>
   </si>
   <si>
@@ -556,7 +559,7 @@
     <t xml:space="preserve">Note: the earlier 72/100 came from an AI review with a different rubric, so compare old vs new on THIS rubric, not against 72.</t>
   </si>
   <si>
-    <t xml:space="preserve">Result used in the deck (1 Nov): the 20-question Day 11 set (new prompt, 4 fresh files) was rated by an AI review, the same kind of review that gave the Day 9 set 72/100. Day 11: 76/100 (17 of 20 questions rated individually). Strong source grounding and scenarios; still weak distractors, longer correct answers, one cross-question clue. Stored answer letters A 35%, B 20%, C 40%, D 5% (the practice page shuffles positions). Next fix: an automatic quality-check step. The rubric below was not used.</t>
+    <t xml:space="preserve">Result used in the deck (1 Nov): the 20-question Day 11 set (new prompt, 4 fresh files) was rated in a separate AI-assisted review, not on the same rubric as the review that gave the Day 9 set 72/100, so the two scores are not directly comparable. Day 11: 76/100 (17 of 20 questions rated individually). Strong source grounding and scenarios; still weak distractors, longer correct answers, one cross-question clue. Stored answer letters A 35%, B 20%, C 40%, D 5% (the practice page shuffles positions). Next fix: an automatic quality-check step. The rubric below was not used.</t>
   </si>
   <si>
     <t xml:space="preserve">Set</t>
@@ -1420,8 +1423,8 @@
         <v>46</v>
       </c>
       <c r="H13" s="1" t="str">
-        <f aca="false">IF(H5=0,"","Manual self-audit (Day 10, by Naw Aung): "&amp;H6&amp;" of "&amp;H5&amp;" claims supported ("&amp;TEXT(H10,"0%")&amp;") across "&amp;H11&amp;" notes (3 case, 5 core) drawn at random by n8n, "&amp;H12&amp;" substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: "&amp;COUNTIF(J15:J44,"Y*")&amp;" of 10 agree. 2 quiz notes in the sample were excluded.")</f>
-        <v>Manual self-audit (Day 10, by Naw Aung): 30 of 30 claims supported (100%) across 8 notes (3 case, 5 core) drawn at random by n8n, 0 substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: 10 of 10 agree. 2 quiz notes in the sample were excluded.</v>
+        <f aca="false">IF(H5=0,"","Manual self-audit (Day 10, by Naw Aung): "&amp;H6&amp;" of "&amp;H5&amp;" claims supported ("&amp;TEXT(H10,"0%")&amp;") across "&amp;H11&amp;" notes (3 case, 5 core) drawn at random by n8n, "&amp;H12&amp;" substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: "&amp;COUNTIF(J15:J44,"Y*")&amp;" of 10 agree (1 rated Interpretation). 2 quiz notes in the sample were excluded.")</f>
+        <v>Manual self-audit (Day 10, by Naw Aung): 30 of 30 claims supported (100%) across 8 notes (3 case, 5 core) drawn at random by n8n, 0 substantive errors; each checked against the source page. 2 classmates blind-checked 10 random claims: 9 of 10 agree (1 rated Interpretation). 2 quiz notes in the sample were excluded.</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2071,7 +2074,7 @@
         <v>61</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2085,7 +2088,7 @@
         <v>67</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E38" s="7" t="s">
         <v>103</v>
@@ -2113,17 +2116,17 @@
         <v>67</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>28</v>
       </c>
       <c r="G39" s="7"/>
       <c r="H39" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I39" s="7" t="s">
         <v>61</v>
@@ -2141,10 +2144,10 @@
         <v>67</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>28</v>
@@ -2160,19 +2163,19 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>81</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>28</v>
@@ -2186,19 +2189,19 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>81</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D42" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E42" s="7" t="s">
         <v>114</v>
-      </c>
-      <c r="E42" s="7" t="s">
-        <v>113</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>28</v>
@@ -2212,19 +2215,19 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>81</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>28</v>
@@ -2238,19 +2241,19 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>81</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>28</v>
@@ -4365,20 +4368,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="11"/>
@@ -4390,10 +4393,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="11"/>
@@ -4405,10 +4408,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C6" s="11"/>
       <c r="D6" s="11"/>
@@ -4420,10 +4423,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C7" s="11"/>
       <c r="D7" s="11"/>
@@ -4435,10 +4438,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C8" s="11"/>
       <c r="D8" s="11"/>
@@ -4450,57 +4453,57 @@
     </row>
     <row r="10" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="L10" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>2061</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F11" s="12" t="n">
         <v>0</v>
@@ -4520,27 +4523,27 @@
         <v>4.20669577874818</v>
       </c>
       <c r="K11" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L11" s="11" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D12" s="11" t="n">
         <v>2360</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>1.02</v>
@@ -4560,27 +4563,27 @@
         <v>0.930084745762712</v>
       </c>
       <c r="K12" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L12" s="11" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D13" s="11" t="n">
         <v>2077</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F13" s="12" t="n">
         <v>0</v>
@@ -4600,27 +4603,27 @@
         <v>3.15358690418873</v>
       </c>
       <c r="K13" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L13" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>1578</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>1.02</v>
@@ -4640,10 +4643,10 @@
         <v>1.39100126742712</v>
       </c>
       <c r="K14" s="11" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="L14" s="11" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4653,7 +4656,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B17" s="15" t="n">
         <f aca="false">IFERROR((H11+H13)/(D11+D13)*1000,"")</f>
@@ -4662,7 +4665,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B18" s="15" t="n">
         <f aca="false">IFERROR((H12+H14)/(D12+D14)*1000,"")</f>
@@ -4671,7 +4674,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B19" s="16" t="n">
         <f aca="false">IFERROR(1-B18/B17,"")</f>
@@ -4680,18 +4683,18 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>2.92</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B21" s="17" t="n">
         <v>0.81</v>
@@ -4699,7 +4702,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B22" s="16" t="n">
         <f aca="false">1-B21/B20</f>
@@ -4754,105 +4757,105 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>171</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L11" s="19" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M11" s="19" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="N11" s="19" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B12" s="6" t="n">
         <v>1</v>
@@ -4869,7 +4872,7 @@
       </c>
       <c r="J12" s="7"/>
       <c r="L12" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="M12" s="8" t="n">
         <f aca="false">SUM(I12:I31)</f>
@@ -4882,7 +4885,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B13" s="6" t="n">
         <v>2</v>
@@ -4899,7 +4902,7 @@
       </c>
       <c r="J13" s="7"/>
       <c r="L13" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="M13" s="8" t="n">
         <f aca="false">SUM(G12:G31)</f>
@@ -4912,7 +4915,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B14" s="6" t="n">
         <v>3</v>
@@ -4929,7 +4932,7 @@
       </c>
       <c r="J14" s="7"/>
       <c r="L14" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="M14" s="8" t="n">
         <f aca="false">SUM(H12:H31)</f>
@@ -4942,7 +4945,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B15" s="6" t="n">
         <v>4</v>
@@ -4959,7 +4962,7 @@
       </c>
       <c r="J15" s="7"/>
       <c r="L15" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M15" s="8" t="n">
         <f aca="false">SUM(E12:E31)</f>
@@ -4972,7 +4975,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B16" s="6" t="n">
         <v>5</v>
@@ -4989,7 +4992,7 @@
       </c>
       <c r="J16" s="7"/>
       <c r="L16" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="M16" s="20" t="str">
         <f aca="false">IFERROR(COUNTIF(D12:D31,"B")/COUNTA(D12:D31),"")</f>
@@ -5002,7 +5005,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B17" s="6" t="n">
         <v>6</v>
@@ -5019,7 +5022,7 @@
       </c>
       <c r="J17" s="7"/>
       <c r="L17" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M17" s="8" t="n">
         <f aca="false">COUNT(I12:I31)</f>
@@ -5032,7 +5035,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B18" s="6" t="n">
         <v>7</v>
@@ -5049,7 +5052,7 @@
       </c>
       <c r="J18" s="7"/>
       <c r="L18" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="M18" s="20" t="str">
         <f aca="false">IFERROR(M12/(M17*5),"")</f>
@@ -5062,7 +5065,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B19" s="6" t="n">
         <v>8</v>
@@ -5081,7 +5084,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B20" s="6" t="n">
         <v>9</v>
@@ -5103,7 +5106,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>10</v>
@@ -5126,7 +5129,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B22" s="6" t="n">
         <v>11</v>
@@ -5145,7 +5148,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B23" s="6" t="n">
         <v>12</v>
@@ -5164,7 +5167,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B24" s="6" t="n">
         <v>13</v>
@@ -5183,7 +5186,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B25" s="6" t="n">
         <v>14</v>
@@ -5202,7 +5205,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B26" s="6" t="n">
         <v>15</v>
@@ -5221,7 +5224,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B27" s="6" t="n">
         <v>16</v>
@@ -5240,7 +5243,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B28" s="6" t="n">
         <v>17</v>
@@ -5259,7 +5262,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B29" s="6" t="n">
         <v>18</v>
@@ -5278,7 +5281,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B30" s="6" t="n">
         <v>19</v>
@@ -5297,7 +5300,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B31" s="6" t="n">
         <v>20</v>
@@ -5316,7 +5319,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B32" s="6" t="n">
         <v>1</v>
@@ -5335,7 +5338,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B33" s="6" t="n">
         <v>2</v>
@@ -5354,7 +5357,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B34" s="6" t="n">
         <v>3</v>
@@ -5373,7 +5376,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B35" s="6" t="n">
         <v>4</v>
@@ -5392,7 +5395,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B36" s="6" t="n">
         <v>5</v>
@@ -5411,7 +5414,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B37" s="6" t="n">
         <v>6</v>
@@ -5430,7 +5433,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B38" s="6" t="n">
         <v>7</v>
@@ -5449,7 +5452,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B39" s="6" t="n">
         <v>8</v>
@@ -5468,7 +5471,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B40" s="6" t="n">
         <v>9</v>
@@ -5487,7 +5490,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B41" s="6" t="n">
         <v>10</v>
@@ -5506,7 +5509,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B42" s="6" t="n">
         <v>11</v>
@@ -5525,7 +5528,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B43" s="6" t="n">
         <v>12</v>
@@ -5544,7 +5547,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B44" s="6" t="n">
         <v>13</v>
@@ -5563,7 +5566,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B45" s="6" t="n">
         <v>14</v>
@@ -5582,7 +5585,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B46" s="6" t="n">
         <v>15</v>
@@ -5601,7 +5604,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B47" s="6" t="n">
         <v>16</v>
@@ -5620,7 +5623,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B48" s="6" t="n">
         <v>17</v>
@@ -5639,7 +5642,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B49" s="6" t="n">
         <v>18</v>
@@ -5658,7 +5661,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B50" s="6" t="n">
         <v>19</v>
@@ -5677,7 +5680,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B51" s="6" t="n">
         <v>20</v>

</xml_diff>